<commit_message>
Daily slate 2026-03-28 [auto]
</commit_message>
<xml_diff>
--- a/Soccer/step8_soccer_direction_clean.xlsx
+++ b/Soccer/step8_soccer_direction_clean.xlsx
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
@@ -3586,21 +3586,21 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Renan Peixoto</t>
+          <t>Alejandro García</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Attacker</t>
+          <t>Midfielder</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -3623,10 +3623,14 @@
           <t>03/29 6:30 PM</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>268187</t>
+        </is>
+      </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Assists</t>
+          <t>Goal + Assist</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
@@ -3651,10 +3655,10 @@
         <v>-0.5</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="S22" s="3" t="inlineStr"/>
       <c r="T22" s="3" t="inlineStr"/>
@@ -3711,17 +3715,17 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Alejandro García</t>
+          <t>Renan Peixoto</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Midfielder</t>
+          <t>Attacker</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>FWD</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -3744,14 +3748,10 @@
           <t>03/29 6:30 PM</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>268187</t>
-        </is>
-      </c>
+      <c r="J23" s="6" t="inlineStr"/>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Goal + Assist</t>
+          <t>Assists</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -3776,10 +3776,10 @@
         <v>-0.5</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="S23" s="6" t="inlineStr"/>
       <c r="T23" s="6" t="inlineStr"/>
@@ -4078,7 +4078,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
@@ -4227,26 +4227,26 @@
         </is>
       </c>
       <c r="B27" s="6" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>Jordan Barrera</t>
+          <t>Steven Mendoza</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>Midfielder</t>
+          <t>Attacker</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>FWD</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>BOTAFOGO</t>
+          <t>ATHLETICO PR</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -4266,12 +4266,12 @@
       </c>
       <c r="J27" s="6" t="inlineStr">
         <is>
-          <t>360063</t>
+          <t>197049</t>
         </is>
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>Shots On Target</t>
+          <t>Goals</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
@@ -4290,25 +4290,25 @@
         </is>
       </c>
       <c r="O27" s="6" t="n">
-        <v>-0.17</v>
+        <v>0</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>0.33</v>
+        <v>0.5</v>
       </c>
       <c r="Q27" s="6" t="n">
-        <v>0.33</v>
+        <v>0.5</v>
       </c>
       <c r="R27" s="6" t="n">
-        <v>0.33</v>
+        <v>0.5</v>
       </c>
       <c r="S27" s="6" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="T27" s="6" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="U27" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V27" s="6" t="n">
         <v>2</v>
@@ -4342,10 +4342,14 @@
       </c>
       <c r="AD27" s="6" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AE27" s="6" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AE27" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="AF27" s="6" t="inlineStr"/>
       <c r="AG27" s="6" t="inlineStr"/>
       <c r="AH27" s="6" t="inlineStr"/>
@@ -4354,7 +4358,7 @@
       <c r="AK27" s="6" t="inlineStr"/>
       <c r="AL27" s="6" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="AM27" s="6" t="inlineStr"/>
@@ -4380,22 +4384,22 @@
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Steven Mendoza</t>
+          <t>Jordan Barrera</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>Attacker</t>
+          <t>Midfielder</t>
         </is>
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>ATHLETICO PR</t>
+          <t>BOTAFOGO</t>
         </is>
       </c>
       <c r="G28" s="3" t="inlineStr">
@@ -4415,12 +4419,12 @@
       </c>
       <c r="J28" s="3" t="inlineStr">
         <is>
-          <t>197049</t>
+          <t>360063</t>
         </is>
       </c>
       <c r="K28" s="3" t="inlineStr">
         <is>
-          <t>Goals</t>
+          <t>Shots On Target</t>
         </is>
       </c>
       <c r="L28" s="3" t="inlineStr">
@@ -4439,25 +4443,25 @@
         </is>
       </c>
       <c r="O28" s="3" t="n">
-        <v>0</v>
+        <v>-0.17</v>
       </c>
       <c r="P28" s="3" t="n">
-        <v>0.5</v>
+        <v>0.33</v>
       </c>
       <c r="Q28" s="3" t="n">
-        <v>0.5</v>
+        <v>0.33</v>
       </c>
       <c r="R28" s="3" t="n">
-        <v>0.5</v>
+        <v>0.33</v>
       </c>
       <c r="S28" s="3" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="T28" s="3" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="U28" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V28" s="3" t="n">
         <v>2</v>
@@ -4491,14 +4495,10 @@
       </c>
       <c r="AD28" s="3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AE28" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE28" s="3" t="inlineStr"/>
       <c r="AF28" s="3" t="inlineStr"/>
       <c r="AG28" s="3" t="inlineStr"/>
       <c r="AH28" s="3" t="inlineStr"/>
@@ -4507,7 +4507,7 @@
       <c r="AK28" s="3" t="inlineStr"/>
       <c r="AL28" s="3" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="AM28" s="3" t="inlineStr"/>
@@ -29115,7 +29115,7 @@
         </is>
       </c>
       <c r="B21" s="6" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
@@ -29240,21 +29240,21 @@
         </is>
       </c>
       <c r="B22" s="3" t="n">
-        <v>0.39</v>
+        <v>0.38</v>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Renan Peixoto</t>
+          <t>Alejandro García</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Attacker</t>
+          <t>Midfielder</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -29277,10 +29277,14 @@
           <t>03/29 6:30 PM</t>
         </is>
       </c>
-      <c r="J22" s="3" t="inlineStr"/>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>268187</t>
+        </is>
+      </c>
       <c r="K22" s="3" t="inlineStr">
         <is>
-          <t>Assists</t>
+          <t>Goal + Assist</t>
         </is>
       </c>
       <c r="L22" s="3" t="inlineStr">
@@ -29305,10 +29309,10 @@
         <v>-0.5</v>
       </c>
       <c r="Q22" s="3" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="R22" s="3" t="n">
-        <v>0.46</v>
+        <v>0.45</v>
       </c>
       <c r="S22" s="3" t="inlineStr"/>
       <c r="T22" s="3" t="inlineStr"/>
@@ -29365,17 +29369,17 @@
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Alejandro García</t>
+          <t>Renan Peixoto</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Midfielder</t>
+          <t>Attacker</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>FWD</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
@@ -29398,14 +29402,10 @@
           <t>03/29 6:30 PM</t>
         </is>
       </c>
-      <c r="J23" s="6" t="inlineStr">
-        <is>
-          <t>268187</t>
-        </is>
-      </c>
+      <c r="J23" s="6" t="inlineStr"/>
       <c r="K23" s="6" t="inlineStr">
         <is>
-          <t>Goal + Assist</t>
+          <t>Assists</t>
         </is>
       </c>
       <c r="L23" s="6" t="inlineStr">
@@ -29430,10 +29430,10 @@
         <v>-0.5</v>
       </c>
       <c r="Q23" s="6" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="R23" s="6" t="n">
-        <v>0.45</v>
+        <v>0.46</v>
       </c>
       <c r="S23" s="6" t="inlineStr"/>
       <c r="T23" s="6" t="inlineStr"/>
@@ -29997,7 +29997,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
@@ -30146,26 +30146,26 @@
         </is>
       </c>
       <c r="B3" s="6" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>Jordan Barrera</t>
+          <t>Steven Mendoza</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
         <is>
-          <t>Midfielder</t>
+          <t>Attacker</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>FWD</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>BOTAFOGO</t>
+          <t>ATHLETICO PR</t>
         </is>
       </c>
       <c r="G3" s="6" t="inlineStr">
@@ -30185,12 +30185,12 @@
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>360063</t>
+          <t>197049</t>
         </is>
       </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>Shots On Target</t>
+          <t>Goals</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
@@ -30209,25 +30209,25 @@
         </is>
       </c>
       <c r="O3" s="6" t="n">
-        <v>-0.17</v>
+        <v>0</v>
       </c>
       <c r="P3" s="6" t="n">
-        <v>0.33</v>
+        <v>0.5</v>
       </c>
       <c r="Q3" s="6" t="n">
-        <v>0.33</v>
+        <v>0.5</v>
       </c>
       <c r="R3" s="6" t="n">
-        <v>0.33</v>
+        <v>0.5</v>
       </c>
       <c r="S3" s="6" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="T3" s="6" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="U3" s="6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V3" s="6" t="n">
         <v>2</v>
@@ -30261,10 +30261,14 @@
       </c>
       <c r="AD3" s="6" t="inlineStr">
         <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="AE3" s="6" t="inlineStr"/>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AE3" s="6" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
       <c r="AF3" s="6" t="inlineStr"/>
       <c r="AG3" s="6" t="inlineStr"/>
       <c r="AH3" s="6" t="inlineStr"/>
@@ -30273,7 +30277,7 @@
       <c r="AK3" s="6" t="inlineStr"/>
       <c r="AL3" s="6" t="inlineStr">
         <is>
-          <t>0.333</t>
+          <t>0.5</t>
         </is>
       </c>
       <c r="AM3" s="6" t="inlineStr"/>
@@ -30299,22 +30303,22 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Steven Mendoza</t>
+          <t>Jordan Barrera</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Attacker</t>
+          <t>Midfielder</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>ATHLETICO PR</t>
+          <t>BOTAFOGO</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -30334,12 +30338,12 @@
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>197049</t>
+          <t>360063</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>Goals</t>
+          <t>Shots On Target</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
@@ -30358,25 +30362,25 @@
         </is>
       </c>
       <c r="O4" s="3" t="n">
-        <v>0</v>
+        <v>-0.17</v>
       </c>
       <c r="P4" s="3" t="n">
-        <v>0.5</v>
+        <v>0.33</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>0.5</v>
+        <v>0.33</v>
       </c>
       <c r="R4" s="3" t="n">
-        <v>0.5</v>
+        <v>0.33</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="U4" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V4" s="3" t="n">
         <v>2</v>
@@ -30410,14 +30414,10 @@
       </c>
       <c r="AD4" s="3" t="inlineStr">
         <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AE4" s="3" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE4" s="3" t="inlineStr"/>
       <c r="AF4" s="3" t="inlineStr"/>
       <c r="AG4" s="3" t="inlineStr"/>
       <c r="AH4" s="3" t="inlineStr"/>
@@ -30426,7 +30426,7 @@
       <c r="AK4" s="3" t="inlineStr"/>
       <c r="AL4" s="3" t="inlineStr">
         <is>
-          <t>0.5</t>
+          <t>0.333</t>
         </is>
       </c>
       <c r="AM4" s="3" t="inlineStr"/>

</xml_diff>